<commit_message>
Wartungsmodus On Off 404 Seite Choräle ausblenden Video fix
</commit_message>
<xml_diff>
--- a/Notenliste.xlsx
+++ b/Notenliste.xlsx
@@ -2191,7 +2191,7 @@
     <t>Tierolff</t>
   </si>
   <si>
-    <t>Südböhmische Polka (2) A4 Format</t>
+    <t>Südböhmische Polka (2)</t>
   </si>
   <si>
     <t>Enzo da Rold</t>
@@ -3589,7 +3589,7 @@
     <t>1150a</t>
   </si>
   <si>
-    <t>Immer voran</t>
+    <t>Frisch voran! (Sempre avanti!)</t>
   </si>
   <si>
     <t>Hans Swistun</t>
@@ -3778,7 +3778,7 @@
     <t>Vladimir Fuka</t>
   </si>
   <si>
-    <t>Südböhmische Polka (1) A5-Format</t>
+    <t>Südböhmische Polka (1)</t>
   </si>
   <si>
     <t>1653a</t>
@@ -4243,7 +4243,7 @@
     <t>Peter Alber</t>
   </si>
   <si>
-    <t>Rock that Beach</t>
+    <t>Rock This Band!</t>
   </si>
   <si>
     <t>Robert Sheldon</t>

</xml_diff>